<commit_message>
update file on 28-08-2026
</commit_message>
<xml_diff>
--- a/1234567.xlsx
+++ b/1234567.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/565755648f0a3f81/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="106" documentId="8_{F92E2664-E68F-4788-901C-B0B3E7C55010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BBA06D6-7BE7-43D8-8E0D-BDD6850B36DA}"/>
+  <xr:revisionPtr revIDLastSave="118" documentId="8_{F92E2664-E68F-4788-901C-B0B3E7C55010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB3056ED-6BC8-45F0-A820-DCEA9BFA1D12}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="63">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1392,26 +1392,50 @@
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+      <c r="A14" s="13">
+        <v>46262</v>
+      </c>
+      <c r="B14" s="14">
+        <v>360</v>
+      </c>
+      <c r="C14" s="14">
+        <v>30</v>
+      </c>
+      <c r="D14" s="14">
+        <v>120</v>
+      </c>
+      <c r="E14" s="14">
+        <v>120</v>
+      </c>
+      <c r="F14" s="14">
+        <v>200</v>
+      </c>
+      <c r="G14" s="14">
+        <v>4</v>
+      </c>
+      <c r="H14" s="14">
+        <v>160</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>990</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="17"/>
+        <v>450</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>

</xml_diff>